<commit_message>
Remove duplicate HorseLuis folder; sync latest edits to root files
</commit_message>
<xml_diff>
--- a/VTT Tool/VTT DATA.xlsx
+++ b/VTT Tool/VTT DATA.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOJorge\Documents\Python projects\Horse Luis\VTT Tool\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\OLMEDOGALVEZJorgeLui\Python Porjects\HorseLuis\VTT Tool\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CF5AAF0-6DCC-40F8-828E-9CE26E0EB6CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{364E7D07-101A-4478-91B4-7969C0CBC0A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1170" yWindow="1170" windowWidth="38700" windowHeight="18780" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" xr2:uid="{7F9BAF1D-C4F9-4C63-99BA-ADCB8DC6383A}"/>
   </bookViews>
   <sheets>
     <sheet name="VTT actif" sheetId="1" r:id="rId1"/>
@@ -754,7 +754,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="781" uniqueCount="180">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="782" uniqueCount="182">
   <si>
     <t>Compte Consignee</t>
   </si>
@@ -1294,6 +1294,12 @@
   </si>
   <si>
     <t>TRYAR</t>
+  </si>
+  <si>
+    <t>Horse Argentina</t>
+  </si>
+  <si>
+    <t>O0012</t>
   </si>
 </sst>
 </file>
@@ -1304,7 +1310,7 @@
     <numFmt numFmtId="164" formatCode="0000000000"/>
     <numFmt numFmtId="165" formatCode="00########"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1503,7 +1509,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -1526,12 +1532,23 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="164" fontId="0" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1682,6 +1699,10 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="15" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2022,10 +2043,10 @@
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
   <dimension ref="A1:BF67"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.42578125" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="9.5703125" customWidth="1"/>
-    <col min="2" max="2" width="10" style="8" customWidth="1"/>
+    <col min="2" max="2" width="17.140625" style="8" customWidth="1"/>
     <col min="3" max="3" width="9.28515625" customWidth="1"/>
     <col min="4" max="4" width="8.7109375" customWidth="1"/>
     <col min="5" max="5" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -2049,7 +2070,7 @@
     <col min="51" max="51" width="13.28515625" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:58" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:58" ht="45" customHeight="1">
       <c r="A1" s="10" t="s">
         <v>5</v>
       </c>
@@ -2216,7 +2237,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58">
       <c r="A2" s="5" t="s">
         <v>138</v>
       </c>
@@ -2323,40 +2344,40 @@
         <v>74</v>
       </c>
       <c r="AI2" s="23">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="AJ2" s="23">
         <f t="shared" ref="AJ2:AJ33" si="6">+AI2+AH2</f>
-        <v>81</v>
+        <v>77</v>
       </c>
       <c r="AK2" s="23"/>
       <c r="AL2" s="23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AM2" s="23">
         <f t="shared" ref="AM2:AM33" si="7">+AJ2+AL2</f>
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="AN2" s="23">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="AO2" s="23">
         <f t="shared" ref="AO2:AO33" si="8">+AM2+AN2</f>
-        <v>89</v>
+        <v>81</v>
       </c>
       <c r="AP2" s="23">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="AQ2" s="3">
-        <v>92</v>
+        <v>84</v>
       </c>
       <c r="AR2" s="23">
-        <f>+AQ2+4</f>
-        <v>96</v>
+        <f>+AQ2+7</f>
+        <v>91</v>
       </c>
       <c r="AS2" s="23">
         <f t="shared" ref="AS2:AS33" si="9">+AR2+7+AT2</f>
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="AT2" s="23">
         <v>14</v>
@@ -2378,7 +2399,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="3" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:58">
       <c r="A3" s="5" t="s">
         <v>171</v>
       </c>
@@ -2541,7 +2562,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="4" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:58">
       <c r="A4" s="5" t="s">
         <v>143</v>
       </c>
@@ -2716,7 +2737,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="5" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:58">
       <c r="A5" s="5" t="s">
         <v>144</v>
       </c>
@@ -2888,7 +2909,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="6" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:58">
       <c r="A6" s="5" t="s">
         <v>145</v>
       </c>
@@ -3061,7 +3082,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="7" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:58">
       <c r="A7" s="5" t="s">
         <v>146</v>
       </c>
@@ -3236,7 +3257,7 @@
         <v>46142</v>
       </c>
     </row>
-    <row r="8" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:58">
       <c r="A8" s="5" t="s">
         <v>147</v>
       </c>
@@ -3408,7 +3429,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="9" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:58">
       <c r="A9" s="5" t="s">
         <v>152</v>
       </c>
@@ -3428,7 +3449,7 @@
         <v>90016000</v>
       </c>
       <c r="G9" s="5" t="s">
-        <v>34</v>
+        <v>180</v>
       </c>
       <c r="H9" s="2">
         <v>0</v>
@@ -3582,7 +3603,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="10" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:58">
       <c r="A10" s="5" t="s">
         <v>168</v>
       </c>
@@ -3744,7 +3765,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="11" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:58">
       <c r="A11" s="5" t="s">
         <v>172</v>
       </c>
@@ -3907,7 +3928,7 @@
         <v>46143</v>
       </c>
     </row>
-    <row r="12" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:58">
       <c r="A12" s="5" t="s">
         <v>175</v>
       </c>
@@ -4074,7 +4095,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="13" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:58" hidden="1">
       <c r="A13" s="5">
         <v>60</v>
       </c>
@@ -4247,7 +4268,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="14" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:58" hidden="1">
       <c r="A14" s="5">
         <v>120</v>
       </c>
@@ -4420,7 +4441,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="15" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:58" hidden="1">
       <c r="A15" s="5">
         <v>121</v>
       </c>
@@ -4593,7 +4614,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="16" spans="1:58" hidden="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:58" hidden="1">
       <c r="A16" s="5">
         <v>233</v>
       </c>
@@ -4766,7 +4787,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="17" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:51" hidden="1">
       <c r="A17" s="5">
         <v>416</v>
       </c>
@@ -4939,7 +4960,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="18" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:51" hidden="1">
       <c r="A18" s="5">
         <v>901</v>
       </c>
@@ -5112,7 +5133,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="19" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:51" hidden="1">
       <c r="A19" s="5">
         <v>904</v>
       </c>
@@ -5285,7 +5306,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="20" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:51" hidden="1">
       <c r="A20" s="5">
         <v>906</v>
       </c>
@@ -5458,7 +5479,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="21" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:51" hidden="1">
       <c r="A21" s="5">
         <v>907</v>
       </c>
@@ -5631,7 +5652,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="22" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:51" hidden="1">
       <c r="A22" s="5">
         <v>908</v>
       </c>
@@ -5803,7 +5824,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="23" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:51" hidden="1">
       <c r="A23" s="5">
         <v>910</v>
       </c>
@@ -5977,7 +5998,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="24" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:51" hidden="1">
       <c r="A24" s="5">
         <v>912</v>
       </c>
@@ -6150,7 +6171,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="25" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:51" hidden="1">
       <c r="A25" s="5">
         <v>915</v>
       </c>
@@ -6322,7 +6343,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="26" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:51" hidden="1">
       <c r="A26" s="5">
         <v>916</v>
       </c>
@@ -6495,7 +6516,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="27" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:51" hidden="1">
       <c r="A27" s="5">
         <v>917</v>
       </c>
@@ -6668,7 +6689,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="28" spans="1:51" ht="15.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:51" ht="15.75" hidden="1" customHeight="1">
       <c r="A28" s="5">
         <v>918</v>
       </c>
@@ -6841,7 +6862,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="29" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:51" hidden="1">
       <c r="A29" s="5">
         <v>920</v>
       </c>
@@ -7014,7 +7035,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="30" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:51" hidden="1">
       <c r="A30" s="5">
         <v>921</v>
       </c>
@@ -7187,7 +7208,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="31" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:51" hidden="1">
       <c r="A31" s="5">
         <v>924</v>
       </c>
@@ -7360,7 +7381,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="32" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:51" hidden="1">
       <c r="A32" s="5">
         <v>925</v>
       </c>
@@ -7533,7 +7554,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="33" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:51" hidden="1">
       <c r="A33" s="5">
         <v>927</v>
       </c>
@@ -7706,7 +7727,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="34" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:51" hidden="1">
       <c r="A34" s="5">
         <v>928</v>
       </c>
@@ -7879,7 +7900,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="35" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:51" hidden="1">
       <c r="A35" s="5">
         <v>930</v>
       </c>
@@ -8051,7 +8072,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="36" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:51" ht="30" hidden="1">
       <c r="A36" s="5">
         <v>931</v>
       </c>
@@ -8224,7 +8245,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="37" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:51" hidden="1">
       <c r="A37" s="5">
         <v>932</v>
       </c>
@@ -8397,7 +8418,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="38" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:51" hidden="1">
       <c r="A38" s="5">
         <v>1039</v>
       </c>
@@ -8570,7 +8591,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="39" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:51" hidden="1">
       <c r="A39" s="5">
         <v>1045</v>
       </c>
@@ -8743,7 +8764,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="40" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:51" hidden="1">
       <c r="A40" s="5">
         <v>1084</v>
       </c>
@@ -8916,7 +8937,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="41" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:51" hidden="1">
       <c r="A41" s="5">
         <v>752</v>
       </c>
@@ -9087,7 +9108,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="42" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:51" hidden="1">
       <c r="A42" s="5">
         <v>761</v>
       </c>
@@ -9257,7 +9278,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="43" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:51" hidden="1">
       <c r="A43" s="5">
         <v>888</v>
       </c>
@@ -9429,7 +9450,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="44" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:51" hidden="1">
       <c r="A44" s="5">
         <v>1005</v>
       </c>
@@ -9601,7 +9622,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="45" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:51" hidden="1">
       <c r="A45" s="5">
         <v>1006</v>
       </c>
@@ -9773,7 +9794,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="46" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:51" hidden="1">
       <c r="A46" s="5">
         <v>1007</v>
       </c>
@@ -9947,7 +9968,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="47" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:51" hidden="1">
       <c r="A47" s="5">
         <v>1009</v>
       </c>
@@ -10119,7 +10140,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="48" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:51" hidden="1">
       <c r="A48" s="5">
         <v>1010</v>
       </c>
@@ -10291,7 +10312,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="49" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:51" hidden="1">
       <c r="A49" s="5">
         <v>1012</v>
       </c>
@@ -10464,7 +10485,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="50" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:51" s="8" customFormat="1" hidden="1">
       <c r="A50" s="5">
         <v>1014</v>
       </c>
@@ -10636,7 +10657,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="51" spans="1:51" s="8" customFormat="1" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:51" s="8" customFormat="1" hidden="1">
       <c r="A51" s="5">
         <v>1015</v>
       </c>
@@ -10808,7 +10829,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="52" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:51" hidden="1">
       <c r="A52" s="5">
         <v>1034</v>
       </c>
@@ -10980,7 +11001,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="53" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:51" hidden="1">
       <c r="A53" s="5">
         <v>1036</v>
       </c>
@@ -11152,7 +11173,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="54" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:51" hidden="1">
       <c r="A54" s="5">
         <v>1037</v>
       </c>
@@ -11324,7 +11345,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="55" spans="1:51" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:51" hidden="1">
       <c r="A55" s="5">
         <v>1040</v>
       </c>
@@ -11496,33 +11517,38 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="57" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:51">
+      <c r="A56" s="51" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="57" spans="1:51">
       <c r="D57" s="41"/>
     </row>
-    <row r="59" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:51">
       <c r="D59" s="42"/>
     </row>
-    <row r="61" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:51">
       <c r="D61" s="41"/>
     </row>
-    <row r="63" spans="1:51" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:51">
       <c r="D63" s="42"/>
     </row>
-    <row r="65" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="4:4">
       <c r="D65" s="41"/>
     </row>
-    <row r="66" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="4:4">
       <c r="D66" s="42"/>
     </row>
-    <row r="67" spans="4:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="4:4">
       <c r="D67" s="42"/>
     </row>
   </sheetData>
   <sheetProtection formatCells="0" formatColumns="0" formatRows="0" sort="0" autoFilter="0"/>
   <autoFilter ref="A1:AY55" xr:uid="{869D9611-F0E3-4A7A-9239-9C1FA0F0C8DA}">
-    <filterColumn colId="0">
+    <filterColumn colId="47">
       <filters>
-        <filter val="908"/>
+        <filter val="Direct"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -11551,9 +11577,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8F7007F1-B98C-4FB4-AD1E-FC672D1A14BF}">
   <sheetPr codeName="Hoja1"/>
   <dimension ref="B2:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="2" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:5">
       <c r="B2" t="s">
         <v>161</v>
       </c>
@@ -11567,7 +11593,7 @@
         <v>163</v>
       </c>
     </row>
-    <row r="3" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:5">
       <c r="B3" t="s">
         <v>164</v>
       </c>
@@ -11581,7 +11607,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="5" spans="2:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:5">
       <c r="B5" t="s">
         <v>167</v>
       </c>
@@ -11594,7 +11620,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20166134-0068-44E4-897C-A3439A6356AD}">
   <dimension ref="D7:H17"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <cols>
     <col min="4" max="5" width="11" customWidth="1"/>
     <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
@@ -11602,7 +11628,7 @@
     <col min="8" max="8" width="11" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="7" spans="4:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="4:8" ht="30">
       <c r="D7" s="31" t="s">
         <v>6</v>
       </c>
@@ -11619,7 +11645,7 @@
         <v>173</v>
       </c>
     </row>
-    <row r="8" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="8" spans="4:8" ht="15.75">
       <c r="D8" s="5" t="s">
         <v>68</v>
       </c>
@@ -11636,7 +11662,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="9" spans="4:8" ht="15.75">
       <c r="D9" s="43" t="s">
         <v>98</v>
       </c>
@@ -11653,7 +11679,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="10" spans="4:8" ht="15.75">
       <c r="D10" s="43" t="s">
         <v>62</v>
       </c>
@@ -11670,7 +11696,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="11" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="11" spans="4:8" ht="15.75">
       <c r="D11" s="43" t="s">
         <v>68</v>
       </c>
@@ -11687,7 +11713,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="12" spans="4:8" ht="15.75">
       <c r="D12" s="23" t="s">
         <v>68</v>
       </c>
@@ -11704,7 +11730,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="13" spans="4:8" ht="15.75">
       <c r="D13" s="23" t="s">
         <v>68</v>
       </c>
@@ -11721,7 +11747,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="14" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="14" spans="4:8" ht="15.75">
       <c r="D14" s="43" t="s">
         <v>52</v>
       </c>
@@ -11738,7 +11764,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="15" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="15" spans="4:8" ht="15.75">
       <c r="D15" s="23" t="s">
         <v>57</v>
       </c>
@@ -11755,7 +11781,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="16" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="16" spans="4:8" ht="15.75">
       <c r="D16" s="43" t="s">
         <v>90</v>
       </c>
@@ -11772,7 +11798,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="17" spans="4:8" ht="15.75" x14ac:dyDescent="0.25">
+    <row r="17" spans="4:8" ht="15.75">
       <c r="D17" s="43" t="s">
         <v>96</v>
       </c>
@@ -11809,9 +11835,9 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A526D049-164C-47D4-96CD-56CBAA0ABF56}">
   <dimension ref="A1:BF3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:58" ht="45" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:58" ht="45" customHeight="1">
       <c r="A1" s="10" t="s">
         <v>5</v>
       </c>
@@ -11978,7 +12004,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="2" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:58">
       <c r="A2" s="5" t="s">
         <v>176</v>
       </c>
@@ -12138,7 +12164,7 @@
         <v>46507</v>
       </c>
     </row>
-    <row r="3" spans="1:58" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:58">
       <c r="A3" s="5" t="s">
         <v>178</v>
       </c>

</xml_diff>